<commit_message>
reports: include larger-unit rows in the category import file
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DMTF5GjS3P9om8RxKa1WuX
</commit_message>
<xml_diff>
--- a/reports/doi-danh-muc-28-10.xlsx
+++ b/reports/doi-danh-muc-28-10.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BT18"/>
+  <dimension ref="A1:BT24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2765,6 +2765,687 @@
         <v>46129.65170297454</v>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Hàng hóa</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Đồ ăn vặt&gt;&gt;Đồ nội địa Trung&gt;&gt;Đồ chay giả mặn (konjac)</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>6931754808649</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>6931754808649</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Mực Chay OKI OKI Sốt Cay 18g</t>
+        </is>
+      </c>
+      <c r="H19" t="n">
+        <v>148148.15</v>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>8%</t>
+        </is>
+      </c>
+      <c r="J19" t="n">
+        <v>160000</v>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>8%</t>
+        </is>
+      </c>
+      <c r="L19" t="n">
+        <v>68385</v>
+      </c>
+      <c r="M19" t="n">
+        <v>0</v>
+      </c>
+      <c r="N19" t="n">
+        <v>0</v>
+      </c>
+      <c r="O19" t="n">
+        <v>0</v>
+      </c>
+      <c r="P19" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q19" t="n">
+        <v>0</v>
+      </c>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>0 ngày</t>
+        </is>
+      </c>
+      <c r="S19" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="T19" t="n">
+        <v>4.95</v>
+      </c>
+      <c r="U19" t="inlineStr">
+        <is>
+          <t>Hộp</t>
+        </is>
+      </c>
+      <c r="V19" t="inlineStr">
+        <is>
+          <t>6931754808595</t>
+        </is>
+      </c>
+      <c r="W19" t="n">
+        <v>20</v>
+      </c>
+      <c r="Y19" t="inlineStr">
+        <is>
+          <t>6931754808595</t>
+        </is>
+      </c>
+      <c r="AA19" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB19" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC19" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD19" t="n">
+        <v>1</v>
+      </c>
+      <c r="AE19" t="n">
+        <v>1</v>
+      </c>
+      <c r="BT19" s="1" t="n">
+        <v>46323.49442878472</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Hàng hóa</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Đồ ăn vặt&gt;&gt;Đồ nội địa Trung&gt;&gt;Đồ chay giả mặn (konjac)</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>6931754808656</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>6931754808656</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Mực Chay OKI OKI Sốt Chua Ngọt 18g</t>
+        </is>
+      </c>
+      <c r="H20" t="n">
+        <v>148148.15</v>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>8%</t>
+        </is>
+      </c>
+      <c r="J20" t="n">
+        <v>160000</v>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>8%</t>
+        </is>
+      </c>
+      <c r="L20" t="n">
+        <v>68385</v>
+      </c>
+      <c r="M20" t="n">
+        <v>0</v>
+      </c>
+      <c r="N20" t="n">
+        <v>0</v>
+      </c>
+      <c r="O20" t="n">
+        <v>0</v>
+      </c>
+      <c r="P20" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q20" t="n">
+        <v>0</v>
+      </c>
+      <c r="R20" t="inlineStr">
+        <is>
+          <t>0 ngày</t>
+        </is>
+      </c>
+      <c r="S20" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="T20" t="n">
+        <v>4.95</v>
+      </c>
+      <c r="U20" t="inlineStr">
+        <is>
+          <t>Hộp</t>
+        </is>
+      </c>
+      <c r="V20" t="inlineStr">
+        <is>
+          <t>6931754808601</t>
+        </is>
+      </c>
+      <c r="W20" t="n">
+        <v>20</v>
+      </c>
+      <c r="Y20" t="inlineStr">
+        <is>
+          <t>6931754808601</t>
+        </is>
+      </c>
+      <c r="AA20" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB20" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC20" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD20" t="n">
+        <v>1</v>
+      </c>
+      <c r="AE20" t="n">
+        <v>1</v>
+      </c>
+      <c r="BT20" s="1" t="n">
+        <v>46323.4925996875</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Hàng hóa</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Đồ ăn vặt&gt;&gt;Snacks&gt;&gt;Snack bắp &amp; phồng</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>SP878081</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Bắp Giòn Vị Wasabi Hainada</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Hàng nội địa Trung</t>
+        </is>
+      </c>
+      <c r="H21" t="n">
+        <v>231481.48</v>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>8%</t>
+        </is>
+      </c>
+      <c r="J21" t="n">
+        <v>250000</v>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>8%</t>
+        </is>
+      </c>
+      <c r="L21" t="n">
+        <v>150000</v>
+      </c>
+      <c r="M21" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="N21" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="O21" t="n">
+        <v>0</v>
+      </c>
+      <c r="P21" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q21" t="n">
+        <v>0</v>
+      </c>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>360 ngày</t>
+        </is>
+      </c>
+      <c r="S21" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="T21" t="n">
+        <v>49999.95</v>
+      </c>
+      <c r="U21" t="inlineStr">
+        <is>
+          <t>Bịch</t>
+        </is>
+      </c>
+      <c r="V21" t="inlineStr">
+        <is>
+          <t>SP878080</t>
+        </is>
+      </c>
+      <c r="W21" t="n">
+        <v>20</v>
+      </c>
+      <c r="Y21" t="inlineStr">
+        <is>
+          <t>SP878080</t>
+        </is>
+      </c>
+      <c r="AA21" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB21" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC21" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD21" t="n">
+        <v>1</v>
+      </c>
+      <c r="AE21" t="n">
+        <v>1</v>
+      </c>
+      <c r="AJ21" t="inlineStr">
+        <is>
+          <t>24072026</t>
+        </is>
+      </c>
+      <c r="AK21" s="1" t="n">
+        <v>46441</v>
+      </c>
+      <c r="AL21" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="BT21" s="1" t="n">
+        <v>46259.71760466435</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Hàng hóa</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Đồ ăn vặt&gt;&gt;Snacks&gt;&gt;Snack bắp &amp; phồng</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>SP878079</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Bắp Giòn Vị Cay Hainada</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Hàng nội địa Trung</t>
+        </is>
+      </c>
+      <c r="H22" t="n">
+        <v>231481.48</v>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>8%</t>
+        </is>
+      </c>
+      <c r="J22" t="n">
+        <v>250000</v>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>8%</t>
+        </is>
+      </c>
+      <c r="L22" t="n">
+        <v>150000</v>
+      </c>
+      <c r="M22" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="N22" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="O22" t="n">
+        <v>0</v>
+      </c>
+      <c r="P22" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q22" t="n">
+        <v>0</v>
+      </c>
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>89 ngày</t>
+        </is>
+      </c>
+      <c r="S22" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="T22" t="n">
+        <v>49999.95</v>
+      </c>
+      <c r="U22" t="inlineStr">
+        <is>
+          <t>Bịch</t>
+        </is>
+      </c>
+      <c r="V22" t="inlineStr">
+        <is>
+          <t>8936241860290</t>
+        </is>
+      </c>
+      <c r="W22" t="n">
+        <v>20</v>
+      </c>
+      <c r="Y22" t="inlineStr">
+        <is>
+          <t>8936241860290</t>
+        </is>
+      </c>
+      <c r="AA22" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB22" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC22" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD22" t="n">
+        <v>1</v>
+      </c>
+      <c r="AE22" t="n">
+        <v>1</v>
+      </c>
+      <c r="AJ22" t="inlineStr">
+        <is>
+          <t>23072026</t>
+        </is>
+      </c>
+      <c r="AK22" s="1" t="n">
+        <v>46440</v>
+      </c>
+      <c r="AL22" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="BT22" s="1" t="n">
+        <v>46259.71595934028</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Hàng hóa</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Đồ ăn vặt&gt;&gt;Snacks&gt;&gt;Snack bắp &amp; phồng</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>SP878078</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Bắp Giòn Nguyên Vị Hainada</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Hàng nội địa Trung</t>
+        </is>
+      </c>
+      <c r="H23" t="n">
+        <v>231481.48</v>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>8%</t>
+        </is>
+      </c>
+      <c r="J23" t="n">
+        <v>250000</v>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>8%</t>
+        </is>
+      </c>
+      <c r="L23" t="n">
+        <v>150000</v>
+      </c>
+      <c r="M23" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="N23" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="O23" t="n">
+        <v>0</v>
+      </c>
+      <c r="P23" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q23" t="n">
+        <v>0</v>
+      </c>
+      <c r="R23" t="inlineStr">
+        <is>
+          <t>89 ngày</t>
+        </is>
+      </c>
+      <c r="S23" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="T23" t="n">
+        <v>49999.95</v>
+      </c>
+      <c r="U23" t="inlineStr">
+        <is>
+          <t>Bịch</t>
+        </is>
+      </c>
+      <c r="V23" t="inlineStr">
+        <is>
+          <t>8936241860276</t>
+        </is>
+      </c>
+      <c r="W23" t="n">
+        <v>20</v>
+      </c>
+      <c r="Y23" t="inlineStr">
+        <is>
+          <t>8936241860276</t>
+        </is>
+      </c>
+      <c r="AA23" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB23" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC23" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD23" t="n">
+        <v>1</v>
+      </c>
+      <c r="AE23" t="n">
+        <v>1</v>
+      </c>
+      <c r="AJ23" t="inlineStr">
+        <is>
+          <t>23072026</t>
+        </is>
+      </c>
+      <c r="AK23" s="1" t="n">
+        <v>46440</v>
+      </c>
+      <c r="AL23" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="BT23" s="1" t="n">
+        <v>46259.71462484953</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Hàng hóa</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Đồ khô - Mì Gói&gt;&gt;Mì trộn / mì khô / spaghetti (Gói)</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>SP877803</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Mì xào Koreno volcano vị gà 118g</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>Koreno</t>
+        </is>
+      </c>
+      <c r="H24" t="n">
+        <v>444444.44</v>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>8%</t>
+        </is>
+      </c>
+      <c r="J24" t="n">
+        <v>480000</v>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>8%</t>
+        </is>
+      </c>
+      <c r="L24" t="n">
+        <v>266666.4</v>
+      </c>
+      <c r="M24" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="N24" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="O24" t="n">
+        <v>0</v>
+      </c>
+      <c r="P24" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q24" t="n">
+        <v>0</v>
+      </c>
+      <c r="R24" t="inlineStr">
+        <is>
+          <t>143 ngày</t>
+        </is>
+      </c>
+      <c r="S24" t="n">
+        <v>0.2083333333333333</v>
+      </c>
+      <c r="T24" t="n">
+        <v>41666666.625</v>
+      </c>
+      <c r="U24" t="inlineStr">
+        <is>
+          <t>Thùng</t>
+        </is>
+      </c>
+      <c r="V24" t="inlineStr">
+        <is>
+          <t>8936028641081</t>
+        </is>
+      </c>
+      <c r="W24" t="n">
+        <v>24</v>
+      </c>
+      <c r="Y24" t="inlineStr">
+        <is>
+          <t>8936028641081</t>
+        </is>
+      </c>
+      <c r="AA24" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB24" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC24" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD24" t="n">
+        <v>1</v>
+      </c>
+      <c r="AE24" t="n">
+        <v>0</v>
+      </c>
+      <c r="BT24" s="1" t="n">
+        <v>46138.09553599537</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>